<commit_message>
Add export functionality for OJT lists and enhance import processes
- Introduced export-ojt-list.php for exporting OJT student data.
- Updated legacy_router.php to include the new export route.
- Enhanced ojt-external-list.php and ojt-internal-list.php to generate export URLs.
- Integrated masterlist import functionality in import-ojt-external.php and import-ojt-internal.php.
- Added ojt_masterlist_import.php for handling masterlist operations.
- Updated import-students-excel.php to support new student number handling.
- Modified database schema to include student_no in relevant tables.
- Improved header validation and data extraction in import functions.
</commit_message>
<xml_diff>
--- a/BioTern/assets/External Students Template.xlsx
+++ b/BioTern/assets/External Students Template.xlsx
@@ -75,19 +75,20 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <dimension ref="A1:J1"/>
+  <dimension ref="A1:K1"/>
   <sheetFormatPr defaultRowHeight="16.5"/>
   <cols>
     <col min="1" max="1" width="18" customWidth="1"/>
-    <col min="2" max="2" width="34" customWidth="1"/>
-    <col min="3" max="3" width="18" customWidth="1"/>
-    <col min="4" max="4" width="14" customWidth="1"/>
-    <col min="5" max="5" width="48" customWidth="1"/>
-    <col min="6" max="6" width="72" customWidth="1"/>
-    <col min="7" max="7" width="34" customWidth="1"/>
-    <col min="8" max="8" width="28" customWidth="1"/>
-    <col min="9" max="9" width="38" customWidth="1"/>
-    <col min="10" max="10" width="16" customWidth="1"/>
+    <col min="2" max="2" width="16" customWidth="1"/>
+    <col min="3" max="3" width="34" customWidth="1"/>
+    <col min="4" max="4" width="18" customWidth="1"/>
+    <col min="5" max="5" width="14" customWidth="1"/>
+    <col min="6" max="6" width="48" customWidth="1"/>
+    <col min="7" max="7" width="72" customWidth="1"/>
+    <col min="8" max="8" width="34" customWidth="1"/>
+    <col min="9" max="9" width="28" customWidth="1"/>
+    <col min="10" max="10" width="38" customWidth="1"/>
+    <col min="11" max="11" width="16" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" ht="18" customHeight="1">
@@ -98,51 +99,56 @@
       </c>
       <c r="B1" t="inlineStr" s="1">
         <is>
-          <t>student_name</t>
+          <t>school_year</t>
         </is>
       </c>
       <c r="C1" t="inlineStr" s="1">
         <is>
-          <t>contact_no</t>
+          <t>student_name</t>
         </is>
       </c>
       <c r="D1" t="inlineStr" s="1">
         <is>
-          <t>section</t>
+          <t>contact_no</t>
         </is>
       </c>
       <c r="E1" t="inlineStr" s="1">
         <is>
-          <t>company_name</t>
+          <t>section</t>
         </is>
       </c>
       <c r="F1" t="inlineStr" s="1">
         <is>
-          <t>company_address</t>
+          <t>company_name</t>
         </is>
       </c>
       <c r="G1" t="inlineStr" s="1">
         <is>
-          <t>supervisor_name</t>
+          <t>company_address</t>
         </is>
       </c>
       <c r="H1" t="inlineStr" s="1">
         <is>
-          <t>supervisor_position</t>
+          <t>supervisor_name</t>
         </is>
       </c>
       <c r="I1" t="inlineStr" s="1">
         <is>
+          <t>supervisor_position</t>
+        </is>
+      </c>
+      <c r="J1" t="inlineStr" s="1">
+        <is>
           <t>company_representative</t>
         </is>
       </c>
-      <c r="J1" t="inlineStr" s="1">
+      <c r="K1" t="inlineStr" s="1">
         <is>
           <t>status</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:J1"/>
+  <autoFilter ref="A1:K1"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
`Updated company management features and templates`
</commit_message>
<xml_diff>
--- a/BioTern/assets/External Students Template.xlsx
+++ b/BioTern/assets/External Students Template.xlsx
@@ -20,41 +20,20 @@
       <name val="Calibri"/>
     </font>
   </fonts>
-  <fills count="3">
+  <fills count="2">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
     </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFD9D9D9"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
   </fills>
-  <borders count="2">
+  <borders count="1">
     <border>
       <left/>
       <right/>
       <top/>
       <bottom/>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color indexed="64"/>
-      </left>
-      <right style="thin">
-        <color indexed="64"/>
-      </right>
-      <top style="thin">
-        <color indexed="64"/>
-      </top>
-      <bottom style="thin">
-        <color indexed="64"/>
-      </bottom>
       <diagonal/>
     </border>
   </borders>
@@ -63,9 +42,7 @@
   </cellStyleXfs>
   <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -75,23 +52,24 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <dimension ref="A1:K1"/>
+  <dimension ref="A1:L1"/>
   <sheetFormatPr defaultRowHeight="16.5"/>
   <cols>
-    <col min="1" max="1" width="18" customWidth="1"/>
+    <col min="1" max="1" width="16" customWidth="1"/>
     <col min="2" max="2" width="16" customWidth="1"/>
-    <col min="3" max="3" width="34" customWidth="1"/>
-    <col min="4" max="4" width="18" customWidth="1"/>
-    <col min="5" max="5" width="14" customWidth="1"/>
-    <col min="6" max="6" width="48" customWidth="1"/>
-    <col min="7" max="7" width="72" customWidth="1"/>
-    <col min="8" max="8" width="34" customWidth="1"/>
-    <col min="9" max="9" width="28" customWidth="1"/>
-    <col min="10" max="10" width="38" customWidth="1"/>
-    <col min="11" max="11" width="16" customWidth="1"/>
+    <col min="3" max="3" width="28" customWidth="1"/>
+    <col min="4" max="4" width="16" customWidth="1"/>
+    <col min="5" max="5" width="18" customWidth="1"/>
+    <col min="6" max="6" width="28" customWidth="1"/>
+    <col min="7" max="7" width="46" customWidth="1"/>
+    <col min="8" max="8" width="28" customWidth="1"/>
+    <col min="9" max="9" width="24" customWidth="1"/>
+    <col min="10" max="10" width="28" customWidth="1"/>
+    <col min="11" max="11" width="26" customWidth="1"/>
+    <col min="12" max="12" width="18" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" ht="18" customHeight="1">
+    <row r="1">
       <c r="A1" t="inlineStr" s="1">
         <is>
           <t>student_no</t>
@@ -144,11 +122,16 @@
       </c>
       <c r="K1" t="inlineStr" s="1">
         <is>
+          <t>company_representative_position</t>
+        </is>
+      </c>
+      <c r="L1" t="inlineStr" s="1">
+        <is>
           <t>status</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:K1"/>
+  <autoFilter ref="A1:L1"/>
 </worksheet>
 </file>
</xml_diff>